<commit_message>
LH-2421 Don't apply column name validation on exsiting columns (#2628)
* Don't apply column name validation on exsiting columns

* Fix spec

* Add spec to verify if column with quotes are removed
</commit_message>
<xml_diff>
--- a/spec/fixtures/files/sheet/valid_file.xlsx
+++ b/spec/fixtures/files/sheet/valid_file.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10911"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rohanpujari/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rohanpujari/tte/psychometrics/spec/fixtures/files/sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5C60C7E-1F44-564B-A48F-038AEAFACB37}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D0CA84D-BC60-2C49-8BE2-C855902E533F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13160" yWindow="660" windowWidth="29960" windowHeight="19360" xr2:uid="{B78FE29B-F531-B745-9689-E11F7FB5D25C}"/>
+    <workbookView xWindow="3640" yWindow="500" windowWidth="29960" windowHeight="19240" xr2:uid="{B78FE29B-F531-B745-9689-E11F7FB5D25C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -48,10 +48,10 @@
     <t>james@cc.com</t>
   </si>
   <si>
-    <t>Text</t>
-  </si>
-  <si>
     <t>Carpenter</t>
+  </si>
+  <si>
+    <t>Markdown</t>
   </si>
 </sst>
 </file>
@@ -435,7 +435,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -443,7 +443,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>